<commit_message>
Update TREE va Detail
</commit_message>
<xml_diff>
--- a/data/DATA_GIAPHA.xlsx
+++ b/data/DATA_GIAPHA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\giapha\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8439511A-58E8-49AD-B994-EC125E2EEFF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51607121-9B80-4238-8CAE-B538BE6D8C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82229A43-EBB1-44A5-B6DE-F008EE3D4237}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{82229A43-EBB1-44A5-B6DE-F008EE3D4237}"/>
   </bookViews>
   <sheets>
     <sheet name="PERSONS" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="508">
   <si>
     <t>Đời</t>
   </si>
@@ -1104,18 +1104,12 @@
     <t>VISIBILITY</t>
   </si>
   <si>
-    <t>avatar.jpg</t>
-  </si>
-  <si>
     <t>public</t>
   </si>
   <si>
     <t>private</t>
   </si>
   <si>
-    <t>avatar2.jpg</t>
-  </si>
-  <si>
     <t>0389195050</t>
   </si>
   <si>
@@ -1567,6 +1561,12 @@
   </si>
   <si>
     <t>images/persons/VA-11.12.jpg</t>
+  </si>
+  <si>
+    <t>images/persons/CAOPHOVA807.jpg</t>
+  </si>
+  <si>
+    <t>Cáo Phó</t>
   </si>
 </sst>
 </file>
@@ -3033,7 +3033,7 @@
         <v>205</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="L30" s="3"/>
       <c r="M30" s="3">
@@ -3066,7 +3066,7 @@
       <c r="I31" s="18"/>
       <c r="J31" s="18"/>
       <c r="K31" s="18" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L31" s="18"/>
       <c r="M31" s="17">
@@ -3101,7 +3101,7 @@
         <v>205</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="L32" s="3"/>
       <c r="M32" s="3">
@@ -3130,7 +3130,7 @@
       <c r="I33" s="18"/>
       <c r="J33" s="18"/>
       <c r="K33" s="18" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="L33" s="18"/>
       <c r="M33" s="17">
@@ -3165,7 +3165,7 @@
         <v>205</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="L34" s="3"/>
       <c r="M34" s="3">
@@ -3196,7 +3196,7 @@
       <c r="I35" s="18"/>
       <c r="J35" s="18"/>
       <c r="K35" s="18" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="L35" s="18"/>
       <c r="M35" s="17">
@@ -3231,7 +3231,7 @@
         <v>205</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="L36" s="3"/>
       <c r="M36" s="3">
@@ -3260,7 +3260,7 @@
       <c r="I37" s="18"/>
       <c r="J37" s="18"/>
       <c r="K37" s="18" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="L37" s="18"/>
       <c r="M37" s="17">
@@ -3293,7 +3293,7 @@
         <v>205</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="L38" s="3" t="s">
         <v>320</v>
@@ -3324,7 +3324,7 @@
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
       <c r="K39" s="18" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="L39" s="18"/>
       <c r="M39" s="17">
@@ -3357,7 +3357,7 @@
         <v>205</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="L40" s="3"/>
       <c r="M40" s="3">
@@ -3394,10 +3394,10 @@
         <v>205</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="M41" s="3">
         <v>8</v>
@@ -3427,7 +3427,7 @@
       <c r="I42" s="18"/>
       <c r="J42" s="18"/>
       <c r="K42" s="18" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="L42" s="18"/>
       <c r="M42" s="17">
@@ -3462,7 +3462,7 @@
         <v>312</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="L43" s="3"/>
       <c r="M43" s="3">
@@ -3491,7 +3491,7 @@
       <c r="I44" s="18"/>
       <c r="J44" s="18"/>
       <c r="K44" s="18" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="L44" s="18"/>
       <c r="M44" s="17">
@@ -3524,7 +3524,7 @@
         <v>312</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="L45" s="3" t="s">
         <v>317</v>
@@ -3555,7 +3555,7 @@
       <c r="I46" s="18"/>
       <c r="J46" s="18"/>
       <c r="K46" s="18" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="L46" s="18"/>
       <c r="M46" s="17">
@@ -3588,7 +3588,7 @@
         <v>312</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="L47" s="3" t="s">
         <v>318</v>
@@ -3619,7 +3619,7 @@
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
       <c r="K48" s="18" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="L48" s="18"/>
       <c r="M48" s="17">
@@ -3654,7 +3654,7 @@
         <v>207</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5">
@@ -3689,7 +3689,7 @@
         <v>207</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5">
@@ -3718,7 +3718,7 @@
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
       <c r="K51" s="18" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="L51" s="18"/>
       <c r="M51" s="17">
@@ -3755,7 +3755,7 @@
         <v>207</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5">
@@ -3786,7 +3786,7 @@
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
       <c r="K53" s="18" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="L53" s="18"/>
       <c r="M53" s="17">
@@ -3823,7 +3823,7 @@
         <v>207</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="L54" s="5"/>
       <c r="M54" s="5">
@@ -3854,7 +3854,7 @@
       <c r="I55" s="18"/>
       <c r="J55" s="18"/>
       <c r="K55" s="18" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="L55" s="18"/>
       <c r="M55" s="17">
@@ -3889,7 +3889,7 @@
         <v>207</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="L56" s="5"/>
       <c r="M56" s="5">
@@ -3918,7 +3918,7 @@
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="18" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="L57" s="18"/>
       <c r="M57" s="17">
@@ -3953,7 +3953,7 @@
         <v>207</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="L58" s="5"/>
       <c r="M58" s="5">
@@ -3984,7 +3984,7 @@
       <c r="I59" s="18"/>
       <c r="J59" s="18"/>
       <c r="K59" s="18" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="L59" s="18"/>
       <c r="M59" s="17">
@@ -4019,7 +4019,7 @@
         <v>207</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5">
@@ -4050,7 +4050,7 @@
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
       <c r="K61" s="18" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="L61" s="18"/>
       <c r="M61" s="17">
@@ -4085,7 +4085,7 @@
         <v>207</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5">
@@ -4114,7 +4114,7 @@
       <c r="I63" s="18"/>
       <c r="J63" s="18"/>
       <c r="K63" s="18" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="L63" s="18"/>
       <c r="M63" s="17">
@@ -4149,7 +4149,7 @@
         <v>208</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="L64" s="5"/>
       <c r="M64" s="5">
@@ -4178,7 +4178,7 @@
       <c r="I65" s="18"/>
       <c r="J65" s="18"/>
       <c r="K65" s="18" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="L65" s="18"/>
       <c r="M65" s="17">
@@ -4213,7 +4213,7 @@
         <v>208</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="L66" s="5"/>
       <c r="M66" s="5">
@@ -4242,7 +4242,7 @@
       <c r="I67" s="18"/>
       <c r="J67" s="18"/>
       <c r="K67" s="18" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="L67" s="18"/>
       <c r="M67" s="17">
@@ -4277,7 +4277,7 @@
         <v>208</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="L68" s="5"/>
       <c r="M68" s="5">
@@ -4306,7 +4306,7 @@
       <c r="I69" s="18"/>
       <c r="J69" s="18"/>
       <c r="K69" s="18" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="L69" s="18"/>
       <c r="M69" s="17">
@@ -4341,7 +4341,7 @@
         <v>208</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="L70" s="5"/>
       <c r="M70" s="5">
@@ -4370,7 +4370,7 @@
       <c r="I71" s="18"/>
       <c r="J71" s="18"/>
       <c r="K71" s="18" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="L71" s="18"/>
       <c r="M71" s="17">
@@ -4405,7 +4405,7 @@
         <v>208</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="L72" s="5"/>
       <c r="M72" s="5">
@@ -4434,7 +4434,7 @@
       <c r="I73" s="18"/>
       <c r="J73" s="18"/>
       <c r="K73" s="18" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="L73" s="18"/>
       <c r="M73" s="17">
@@ -4469,7 +4469,7 @@
         <v>208</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="L74" s="5"/>
       <c r="M74" s="5">
@@ -4500,7 +4500,7 @@
       <c r="I75" s="18"/>
       <c r="J75" s="18"/>
       <c r="K75" s="18" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="L75" s="18"/>
       <c r="M75" s="17">
@@ -4535,7 +4535,7 @@
         <v>212</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="L76" s="5"/>
       <c r="M76" s="5">
@@ -4566,7 +4566,7 @@
       <c r="I77" s="18"/>
       <c r="J77" s="18"/>
       <c r="K77" s="18" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="L77" s="18"/>
       <c r="M77" s="17">
@@ -4601,7 +4601,7 @@
         <v>212</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="L78" s="5"/>
       <c r="M78" s="5">
@@ -4630,7 +4630,7 @@
       <c r="I79" s="18"/>
       <c r="J79" s="18"/>
       <c r="K79" s="18" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="L79" s="18"/>
       <c r="M79" s="17">
@@ -4665,7 +4665,7 @@
         <v>213</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="L80" s="5"/>
       <c r="M80" s="5">
@@ -4694,7 +4694,7 @@
       <c r="I81" s="18"/>
       <c r="J81" s="18"/>
       <c r="K81" s="18" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="L81" s="18"/>
       <c r="M81" s="17">
@@ -4729,7 +4729,7 @@
         <v>213</v>
       </c>
       <c r="K82" s="22" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="L82" s="22"/>
       <c r="M82" s="22">
@@ -4758,7 +4758,7 @@
       <c r="I83" s="10"/>
       <c r="J83" s="10"/>
       <c r="K83" s="10" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="L83" s="10"/>
       <c r="M83" s="9">
@@ -4793,7 +4793,7 @@
         <v>213</v>
       </c>
       <c r="K84" s="8" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="L84" s="8"/>
       <c r="M84" s="8">
@@ -4822,7 +4822,7 @@
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
       <c r="K85" s="10" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="L85" s="10"/>
       <c r="M85" s="9">
@@ -4855,7 +4855,7 @@
         <v>213</v>
       </c>
       <c r="K86" s="8" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="L86" s="8" t="s">
         <v>308</v>
@@ -4892,7 +4892,7 @@
         <v>217</v>
       </c>
       <c r="K87" s="6" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="L87" s="6"/>
       <c r="M87" s="6">
@@ -4923,7 +4923,7 @@
       <c r="I88" s="10"/>
       <c r="J88" s="10"/>
       <c r="K88" s="10" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="L88" s="10"/>
       <c r="M88" s="9">
@@ -4958,7 +4958,7 @@
         <v>217</v>
       </c>
       <c r="K89" s="6" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="L89" s="6"/>
       <c r="M89" s="6">
@@ -4989,7 +4989,7 @@
       <c r="I90" s="10"/>
       <c r="J90" s="10"/>
       <c r="K90" s="10" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="L90" s="10"/>
       <c r="M90" s="9">
@@ -5020,7 +5020,7 @@
       <c r="I91" s="10"/>
       <c r="J91" s="10"/>
       <c r="K91" s="10" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="L91" s="10" t="s">
         <v>302</v>
@@ -5057,7 +5057,7 @@
         <v>217</v>
       </c>
       <c r="K92" s="6" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="L92" s="6"/>
       <c r="M92" s="6">
@@ -5088,7 +5088,7 @@
       <c r="I93" s="10"/>
       <c r="J93" s="10"/>
       <c r="K93" s="10" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="L93" s="10"/>
       <c r="M93" s="9">
@@ -5123,7 +5123,7 @@
         <v>218</v>
       </c>
       <c r="K94" s="6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="L94" s="6"/>
       <c r="M94" s="6">
@@ -5154,7 +5154,7 @@
       <c r="I95" s="10"/>
       <c r="J95" s="10"/>
       <c r="K95" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="L95" s="10"/>
       <c r="M95" s="9">
@@ -5189,7 +5189,7 @@
         <v>218</v>
       </c>
       <c r="K96" s="6" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="L96" s="6"/>
       <c r="M96" s="6">
@@ -5220,7 +5220,7 @@
       <c r="I97" s="10"/>
       <c r="J97" s="10"/>
       <c r="K97" s="10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="L97" s="10"/>
       <c r="M97" s="9">
@@ -5255,7 +5255,7 @@
         <v>221</v>
       </c>
       <c r="K98" s="6" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="L98" s="6"/>
       <c r="M98" s="6">
@@ -5286,7 +5286,7 @@
       <c r="I99" s="10"/>
       <c r="J99" s="10"/>
       <c r="K99" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="L99" s="10"/>
       <c r="M99" s="9">
@@ -5321,7 +5321,7 @@
         <v>221</v>
       </c>
       <c r="K100" s="6" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="L100" s="6"/>
       <c r="M100" s="6">
@@ -5356,7 +5356,7 @@
         <v>223</v>
       </c>
       <c r="K101" s="6" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="L101" s="6"/>
       <c r="M101" s="6">
@@ -5387,7 +5387,7 @@
       <c r="I102" s="10"/>
       <c r="J102" s="10"/>
       <c r="K102" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="L102" s="10"/>
       <c r="M102" s="9">
@@ -5422,7 +5422,7 @@
         <v>223</v>
       </c>
       <c r="K103" s="6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="L103" s="6"/>
       <c r="M103" s="6">
@@ -5453,7 +5453,7 @@
       <c r="I104" s="10"/>
       <c r="J104" s="10"/>
       <c r="K104" s="10" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="L104" s="10"/>
       <c r="M104" s="9">
@@ -5488,7 +5488,7 @@
         <v>223</v>
       </c>
       <c r="K105" s="6" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="L105" s="6"/>
       <c r="M105" s="6">
@@ -5519,7 +5519,7 @@
       <c r="I106" s="10"/>
       <c r="J106" s="10"/>
       <c r="K106" s="10" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="L106" s="10"/>
       <c r="M106" s="9">
@@ -5554,7 +5554,7 @@
         <v>224</v>
       </c>
       <c r="K107" s="6" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="L107" s="6"/>
       <c r="M107" s="6">
@@ -5585,7 +5585,7 @@
       <c r="I108" s="10"/>
       <c r="J108" s="10"/>
       <c r="K108" s="10" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="L108" s="10"/>
       <c r="M108" s="9">
@@ -5620,7 +5620,7 @@
         <v>224</v>
       </c>
       <c r="K109" s="6" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="L109" s="6"/>
       <c r="M109" s="6">
@@ -5655,7 +5655,7 @@
         <v>228</v>
       </c>
       <c r="K110" s="6" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="L110" s="6"/>
       <c r="M110" s="6">
@@ -5690,7 +5690,7 @@
         <v>228</v>
       </c>
       <c r="K111" s="6" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="L111" s="6"/>
       <c r="M111" s="6">
@@ -5725,7 +5725,7 @@
         <v>229</v>
       </c>
       <c r="K112" s="6" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="L112" s="6"/>
       <c r="M112" s="6">
@@ -5760,7 +5760,7 @@
         <v>229</v>
       </c>
       <c r="K113" s="6" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="L113" s="6"/>
       <c r="M113" s="6">
@@ -5793,7 +5793,7 @@
         <v>231</v>
       </c>
       <c r="K114" s="6" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="L114" s="6"/>
       <c r="M114" s="6">
@@ -5826,7 +5826,7 @@
         <v>231</v>
       </c>
       <c r="K115" s="6" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="L115" s="6"/>
       <c r="M115" s="6">
@@ -5861,7 +5861,7 @@
         <v>232</v>
       </c>
       <c r="K116" s="6" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="L116" s="6"/>
       <c r="M116" s="6">
@@ -5894,7 +5894,7 @@
         <v>232</v>
       </c>
       <c r="K117" s="6" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="L117" s="6"/>
       <c r="M117" s="6">
@@ -5927,7 +5927,7 @@
         <v>232</v>
       </c>
       <c r="K118" s="6" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="L118" s="6"/>
       <c r="M118" s="6">
@@ -5962,7 +5962,7 @@
         <v>234</v>
       </c>
       <c r="K119" s="6" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="L119" s="6"/>
       <c r="M119" s="6">
@@ -5997,7 +5997,7 @@
         <v>234</v>
       </c>
       <c r="K120" s="6" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="L120" s="6"/>
       <c r="M120" s="6">
@@ -6029,10 +6029,10 @@
         <v>68</v>
       </c>
       <c r="J121" s="6" t="s">
-        <v>235</v>
+        <v>300</v>
       </c>
       <c r="K121" s="6" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="L121" s="6"/>
       <c r="M121" s="6">
@@ -6067,7 +6067,7 @@
         <v>235</v>
       </c>
       <c r="K122" s="6" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="L122" s="6"/>
       <c r="M122" s="6">
@@ -6102,7 +6102,7 @@
         <v>237</v>
       </c>
       <c r="K123" s="6" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="L123" s="6"/>
       <c r="M123" s="6">
@@ -6137,7 +6137,7 @@
         <v>237</v>
       </c>
       <c r="K124" s="6" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="L124" s="6"/>
       <c r="M124" s="6">
@@ -6172,7 +6172,7 @@
         <v>240</v>
       </c>
       <c r="K125" s="6" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="L125" s="6"/>
       <c r="M125" s="6">
@@ -6207,7 +6207,7 @@
         <v>240</v>
       </c>
       <c r="K126" s="6" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="L126" s="6"/>
       <c r="M126" s="6">
@@ -6238,7 +6238,7 @@
       <c r="I127" s="10"/>
       <c r="J127" s="10"/>
       <c r="K127" s="13" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="L127" s="10"/>
       <c r="M127" s="9">
@@ -6273,7 +6273,7 @@
         <v>242</v>
       </c>
       <c r="K128" s="6" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="L128" s="6"/>
       <c r="M128" s="6">
@@ -6308,7 +6308,7 @@
         <v>242</v>
       </c>
       <c r="K129" s="6" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="L129" s="6"/>
       <c r="M129" s="6">
@@ -6343,7 +6343,7 @@
         <v>243</v>
       </c>
       <c r="K130" s="6" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="L130" s="6"/>
       <c r="M130" s="6">
@@ -6378,7 +6378,7 @@
         <v>243</v>
       </c>
       <c r="K131" s="6" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="L131" s="6"/>
       <c r="M131" s="6">
@@ -6481,7 +6481,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>202</v>
@@ -6496,7 +6496,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B7" s="24" t="s">
         <v>31</v>
@@ -6512,7 +6512,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B8" s="24" t="s">
         <v>34</v>
@@ -6529,7 +6529,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>34</v>
@@ -6546,7 +6546,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>36</v>
@@ -6561,7 +6561,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B11" s="24" t="s">
         <v>37</v>
@@ -6576,7 +6576,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B12" s="24" t="s">
         <v>38</v>
@@ -6591,7 +6591,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B13" s="24" t="s">
         <v>42</v>
@@ -6606,7 +6606,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B14" s="24" t="s">
         <v>43</v>
@@ -6621,7 +6621,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B15" s="24" t="s">
         <v>48</v>
@@ -6636,7 +6636,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B16" s="24" t="s">
         <v>49</v>
@@ -6651,7 +6651,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B17" s="24" t="s">
         <v>52</v>
@@ -6666,7 +6666,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B18" s="24" t="s">
         <v>54</v>
@@ -6681,7 +6681,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B19" s="24" t="s">
         <v>55</v>
@@ -6696,7 +6696,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B20" s="24" t="s">
         <v>59</v>
@@ -6711,7 +6711,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B21" s="24" t="s">
         <v>60</v>
@@ -6726,7 +6726,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B22" s="24" t="s">
         <v>62</v>
@@ -6741,7 +6741,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B23" s="24" t="s">
         <v>63</v>
@@ -6756,7 +6756,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B24" s="24" t="s">
         <v>66</v>
@@ -6771,7 +6771,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B25" s="24" t="s">
         <v>68</v>
@@ -6788,7 +6788,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="B26" s="24" t="s">
         <v>68</v>
@@ -6805,7 +6805,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="B27" s="24" t="s">
         <v>70</v>
@@ -6820,7 +6820,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B28" s="24" t="s">
         <v>76</v>
@@ -6835,7 +6835,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="B29" s="24" t="s">
         <v>78</v>
@@ -6850,7 +6850,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B30" s="24" t="s">
         <v>80</v>
@@ -6865,7 +6865,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B31" s="24" t="s">
         <v>304</v>
@@ -6905,13 +6905,13 @@
         <v>327</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D1" s="25" t="s">
         <v>328</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -6922,13 +6922,13 @@
         <v>329</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>388</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -6945,7 +6945,7 @@
         <v>331</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -6956,13 +6956,13 @@
         <v>329</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -6973,13 +6973,13 @@
         <v>329</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -6990,13 +6990,13 @@
         <v>329</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -7007,13 +7007,13 @@
         <v>329</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -7030,7 +7030,7 @@
         <v>333</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -7084,16 +7084,16 @@
         <v>68</v>
       </c>
       <c r="B2" s="23" t="s">
+        <v>355</v>
+      </c>
+      <c r="C2" t="s">
+        <v>356</v>
+      </c>
+      <c r="D2" t="s">
         <v>357</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>358</v>
-      </c>
-      <c r="D2" t="s">
-        <v>359</v>
-      </c>
-      <c r="E2" t="s">
-        <v>360</v>
       </c>
     </row>
   </sheetData>
@@ -7103,13 +7103,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2870D094-0F04-43A9-85F0-3281621B51DF}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.140625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7118,13 +7118,13 @@
         <v>350</v>
       </c>
       <c r="B1" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C1" t="s">
         <v>351</v>
       </c>
       <c r="D1" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E1" t="s">
         <v>352</v>
@@ -7135,16 +7135,16 @@
         <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>402</v>
-      </c>
-      <c r="C2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="D2" t="s">
+        <v>401</v>
+      </c>
+      <c r="E2" t="s">
         <v>353</v>
-      </c>
-      <c r="D2" t="s">
-        <v>403</v>
-      </c>
-      <c r="E2" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -7152,16 +7152,67 @@
         <v>68</v>
       </c>
       <c r="B3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="D3" t="s">
         <v>402</v>
       </c>
-      <c r="C3" t="s">
-        <v>356</v>
-      </c>
-      <c r="D3" t="s">
-        <v>404</v>
-      </c>
       <c r="E3" t="s">
-        <v>355</v>
+        <v>354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>400</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="D4" t="s">
+        <v>401</v>
+      </c>
+      <c r="E4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>400</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="D5" t="s">
+        <v>402</v>
+      </c>
+      <c r="E5" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>400</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="D6" t="s">
+        <v>507</v>
+      </c>
+      <c r="E6" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update anh thanh vien
</commit_message>
<xml_diff>
--- a/data/DATA_GIAPHA.xlsx
+++ b/data/DATA_GIAPHA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\giapha\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79CEC64B-D87A-45E5-8F22-57654E008A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2FA415-BBA5-4729-9005-DBC981CC408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{82229A43-EBB1-44A5-B6DE-F008EE3D4237}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1123" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="559">
   <si>
     <t>Đời</t>
   </si>
@@ -1248,12 +1248,6 @@
     <t>images/persons/VA-8.05.jpg</t>
   </si>
   <si>
-    <t>images/persons/VA-8.05S1.jpg</t>
-  </si>
-  <si>
-    <t>images/persons/VA-8.06.jpg</t>
-  </si>
-  <si>
     <t>images/persons/VA-8.07.jpg</t>
   </si>
   <si>
@@ -1263,9 +1257,6 @@
     <t>images/persons/VA-8.08.jpg</t>
   </si>
   <si>
-    <t>images/persons/VA-8.08S1.jpg</t>
-  </si>
-  <si>
     <t>images/persons/VA-8.09.jpg</t>
   </si>
   <si>
@@ -1368,9 +1359,6 @@
     <t>images/persons/VA-9.16.jpg</t>
   </si>
   <si>
-    <t>images/persons/VA-9.16S1.jpg</t>
-  </si>
-  <si>
     <t>images/persons/VA-9.17.jpg</t>
   </si>
   <si>
@@ -1389,9 +1377,6 @@
     <t>images/persons/VA-9.19S1.jpg</t>
   </si>
   <si>
-    <t>images/persons/VA-9.20.jpg</t>
-  </si>
-  <si>
     <t>images/persons/VA-10.01.jpg</t>
   </si>
   <si>
@@ -1404,9 +1389,6 @@
     <t>images/persons/VA-10.02S1.jpg</t>
   </si>
   <si>
-    <t>images/persons/VA-10.02S2.jpg</t>
-  </si>
-  <si>
     <t>images/persons/VA-10.03.jpg</t>
   </si>
   <si>
@@ -1720,6 +1702,24 @@
   </si>
   <si>
     <t>Bắt tay giữa Xuân Đông và Xuân Trường</t>
+  </si>
+  <si>
+    <t>Trần</t>
+  </si>
+  <si>
+    <t>Chanh</t>
+  </si>
+  <si>
+    <t>images/ConTraiVA.jpg</t>
+  </si>
+  <si>
+    <t>images/MoToVA.jpg</t>
+  </si>
+  <si>
+    <t>Ảnh Mộ Tổ Phúc Bằng</t>
+  </si>
+  <si>
+    <t>Tập thể Nam</t>
   </si>
 </sst>
 </file>
@@ -1908,7 +1908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1936,12 +1936,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2335,7 +2333,9 @@
         <v>8</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2">
+        <v>1900</v>
+      </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -2364,7 +2364,9 @@
         <v>11</v>
       </c>
       <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
+      <c r="H3" s="19">
+        <v>1900</v>
+      </c>
       <c r="I3" s="19"/>
       <c r="J3" s="19"/>
       <c r="K3" s="19"/>
@@ -2393,7 +2395,9 @@
         <v>8</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2">
+        <v>1900</v>
+      </c>
       <c r="I4" s="2" t="s">
         <v>6</v>
       </c>
@@ -2424,7 +2428,9 @@
         <v>11</v>
       </c>
       <c r="G5" s="19"/>
-      <c r="H5" s="18"/>
+      <c r="H5" s="18">
+        <v>1900</v>
+      </c>
       <c r="I5" s="18"/>
       <c r="J5" s="18"/>
       <c r="K5" s="18"/>
@@ -2453,7 +2459,9 @@
         <v>8</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2">
+        <v>1900</v>
+      </c>
       <c r="I6" s="2" t="s">
         <v>6</v>
       </c>
@@ -2486,12 +2494,14 @@
         <v>11</v>
       </c>
       <c r="G7" s="19"/>
-      <c r="H7" s="18"/>
+      <c r="H7" s="18">
+        <v>1900</v>
+      </c>
       <c r="I7" s="18"/>
       <c r="J7" s="18"/>
       <c r="K7" s="18"/>
       <c r="L7" s="18" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="M7" s="17">
         <v>5</v>
@@ -2517,7 +2527,9 @@
         <v>8</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="2">
+        <v>1900</v>
+      </c>
       <c r="I8" s="2" t="s">
         <v>6</v>
       </c>
@@ -2526,7 +2538,7 @@
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>533</v>
+        <v>527</v>
       </c>
       <c r="M8" s="2">
         <v>5</v>
@@ -2550,7 +2562,9 @@
         <v>11</v>
       </c>
       <c r="G9" s="19"/>
-      <c r="H9" s="18"/>
+      <c r="H9" s="18">
+        <v>1900</v>
+      </c>
       <c r="I9" s="18"/>
       <c r="J9" s="18"/>
       <c r="K9" s="18"/>
@@ -2579,7 +2593,9 @@
         <v>8</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2">
+        <v>1900</v>
+      </c>
       <c r="I10" s="2" t="s">
         <v>6</v>
       </c>
@@ -2614,7 +2630,9 @@
         <v>8</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="H11" s="2">
+        <v>1900</v>
+      </c>
       <c r="I11" s="2" t="s">
         <v>6</v>
       </c>
@@ -2649,7 +2667,9 @@
         <v>8</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="2">
+        <v>1900</v>
+      </c>
       <c r="I12" s="2" t="s">
         <v>6</v>
       </c>
@@ -2658,7 +2678,7 @@
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="M12" s="2">
         <v>5</v>
@@ -2684,7 +2704,9 @@
         <v>11</v>
       </c>
       <c r="G13" s="19"/>
-      <c r="H13" s="18"/>
+      <c r="H13" s="18">
+        <v>1900</v>
+      </c>
       <c r="I13" s="18"/>
       <c r="J13" s="18"/>
       <c r="K13" s="18"/>
@@ -2713,7 +2735,9 @@
         <v>8</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="H14" s="2">
+        <v>1900</v>
+      </c>
       <c r="I14" s="2" t="s">
         <v>12</v>
       </c>
@@ -2748,7 +2772,9 @@
         <v>8</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2">
+        <v>1900</v>
+      </c>
       <c r="I15" s="2" t="s">
         <v>12</v>
       </c>
@@ -2781,7 +2807,9 @@
         <v>11</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="2">
+        <v>1900</v>
+      </c>
       <c r="I16" s="2" t="s">
         <v>12</v>
       </c>
@@ -2814,7 +2842,9 @@
         <v>8</v>
       </c>
       <c r="G17" s="19"/>
-      <c r="H17" s="18"/>
+      <c r="H17" s="18">
+        <v>1900</v>
+      </c>
       <c r="I17" s="18"/>
       <c r="J17" s="18"/>
       <c r="K17" s="18"/>
@@ -2841,7 +2871,9 @@
         <v>11</v>
       </c>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+      <c r="H18" s="2">
+        <v>1900</v>
+      </c>
       <c r="I18" s="2" t="s">
         <v>16</v>
       </c>
@@ -2872,7 +2904,9 @@
         <v>8</v>
       </c>
       <c r="G19" s="19"/>
-      <c r="H19" s="18"/>
+      <c r="H19" s="18">
+        <v>1900</v>
+      </c>
       <c r="I19" s="18"/>
       <c r="J19" s="18"/>
       <c r="K19" s="18"/>
@@ -2895,13 +2929,15 @@
         <v>124</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>503</v>
+        <v>497</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2">
+        <v>1900</v>
+      </c>
       <c r="I20" s="2" t="s">
         <v>22</v>
       </c>
@@ -2910,7 +2946,7 @@
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="M20" s="2">
         <v>6</v>
@@ -2924,22 +2960,24 @@
         <v>203</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
       <c r="E21" s="19"/>
       <c r="F21" s="17" t="s">
         <v>11</v>
       </c>
       <c r="G21" s="19"/>
-      <c r="H21" s="18"/>
+      <c r="H21" s="18">
+        <v>1900</v>
+      </c>
       <c r="I21" s="18"/>
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
       <c r="L21" s="18" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="M21" s="17">
         <v>6</v>
@@ -2963,7 +3001,9 @@
         <v>8</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
+      <c r="H22" s="2">
+        <v>1900</v>
+      </c>
       <c r="I22" s="2" t="s">
         <v>22</v>
       </c>
@@ -2995,7 +3035,9 @@
         <v>11</v>
       </c>
       <c r="G23" s="19"/>
-      <c r="H23" s="18"/>
+      <c r="H23" s="18">
+        <v>1900</v>
+      </c>
       <c r="I23" s="18"/>
       <c r="J23" s="18"/>
       <c r="K23" s="18"/>
@@ -3022,7 +3064,9 @@
         <v>11</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
+      <c r="H24" s="2">
+        <v>1900</v>
+      </c>
       <c r="I24" s="2" t="s">
         <v>202</v>
       </c>
@@ -3049,7 +3093,7 @@
         <v>126</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>8</v>
@@ -3069,7 +3113,7 @@
       </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="M25" s="2">
         <v>7</v>
@@ -3098,7 +3142,7 @@
       <c r="J26" s="18"/>
       <c r="K26" s="18"/>
       <c r="L26" s="18" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="M26" s="17">
         <v>7</v>
@@ -3131,7 +3175,7 @@
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
       <c r="L27" s="18" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="M27" s="17">
         <v>7</v>
@@ -3212,7 +3256,7 @@
         <v>128</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>8</v>
@@ -3284,7 +3328,7 @@
         <v>129</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>506</v>
+        <v>500</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>8</v>
@@ -3350,7 +3394,7 @@
         <v>130</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>507</v>
+        <v>501</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>8</v>
@@ -3418,7 +3462,7 @@
         <v>131</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>8</v>
@@ -3437,7 +3481,7 @@
         <v>398</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
       <c r="M36" s="3">
         <v>8</v>
@@ -3528,9 +3572,7 @@
       <c r="H39" s="18"/>
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
-      <c r="K39" s="18" t="s">
-        <v>401</v>
-      </c>
+      <c r="K39" s="18"/>
       <c r="L39" s="18"/>
       <c r="M39" s="17">
         <v>8</v>
@@ -3561,9 +3603,7 @@
       <c r="J40" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="K40" s="3" t="s">
-        <v>402</v>
-      </c>
+      <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3">
         <v>8</v>
@@ -3599,7 +3639,7 @@
         <v>205</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>391</v>
@@ -3632,7 +3672,7 @@
       <c r="I42" s="18"/>
       <c r="J42" s="18"/>
       <c r="K42" s="18" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="L42" s="18"/>
       <c r="M42" s="17">
@@ -3667,7 +3707,7 @@
         <v>310</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L43" s="3"/>
       <c r="M43" s="3">
@@ -3695,9 +3735,7 @@
       <c r="H44" s="18"/>
       <c r="I44" s="18"/>
       <c r="J44" s="18"/>
-      <c r="K44" s="18" t="s">
-        <v>406</v>
-      </c>
+      <c r="K44" s="18"/>
       <c r="L44" s="18"/>
       <c r="M44" s="17">
         <v>8</v>
@@ -3729,7 +3767,7 @@
         <v>310</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="L45" s="3" t="s">
         <v>314</v>
@@ -3760,7 +3798,7 @@
       <c r="I46" s="18"/>
       <c r="J46" s="18"/>
       <c r="K46" s="18" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="L46" s="18"/>
       <c r="M46" s="17">
@@ -3793,7 +3831,7 @@
         <v>310</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="L47" s="3" t="s">
         <v>315</v>
@@ -3824,7 +3862,7 @@
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
       <c r="K48" s="18" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="L48" s="18"/>
       <c r="M48" s="17">
@@ -3859,7 +3897,7 @@
         <v>207</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5">
@@ -3894,7 +3932,7 @@
         <v>207</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5">
@@ -3923,7 +3961,7 @@
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
       <c r="K51" s="18" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="L51" s="18"/>
       <c r="M51" s="17">
@@ -3960,7 +3998,7 @@
         <v>207</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5">
@@ -3991,7 +4029,7 @@
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
       <c r="K53" s="18" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="L53" s="18"/>
       <c r="M53" s="17">
@@ -4028,7 +4066,7 @@
         <v>207</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="L54" s="5"/>
       <c r="M54" s="5">
@@ -4059,7 +4097,7 @@
       <c r="I55" s="18"/>
       <c r="J55" s="18"/>
       <c r="K55" s="18" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="L55" s="18"/>
       <c r="M55" s="17">
@@ -4094,7 +4132,7 @@
         <v>207</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="L56" s="5"/>
       <c r="M56" s="5">
@@ -4123,7 +4161,7 @@
       <c r="I57" s="18"/>
       <c r="J57" s="18"/>
       <c r="K57" s="18" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="L57" s="18"/>
       <c r="M57" s="17">
@@ -4158,7 +4196,7 @@
         <v>207</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="L58" s="5"/>
       <c r="M58" s="5">
@@ -4189,7 +4227,7 @@
       <c r="I59" s="18"/>
       <c r="J59" s="18"/>
       <c r="K59" s="18" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="L59" s="18"/>
       <c r="M59" s="17">
@@ -4224,7 +4262,7 @@
         <v>207</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5">
@@ -4255,7 +4293,7 @@
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
       <c r="K61" s="18" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="L61" s="18"/>
       <c r="M61" s="17">
@@ -4290,7 +4328,7 @@
         <v>207</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5">
@@ -4319,7 +4357,7 @@
       <c r="I63" s="18"/>
       <c r="J63" s="18"/>
       <c r="K63" s="18" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="L63" s="18"/>
       <c r="M63" s="17">
@@ -4354,7 +4392,7 @@
         <v>208</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="L64" s="5"/>
       <c r="M64" s="5">
@@ -4383,7 +4421,7 @@
       <c r="I65" s="18"/>
       <c r="J65" s="18"/>
       <c r="K65" s="18" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="L65" s="18"/>
       <c r="M65" s="17">
@@ -4418,7 +4456,7 @@
         <v>208</v>
       </c>
       <c r="K66" s="5" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="L66" s="5"/>
       <c r="M66" s="5">
@@ -4447,7 +4485,7 @@
       <c r="I67" s="18"/>
       <c r="J67" s="18"/>
       <c r="K67" s="18" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="L67" s="18"/>
       <c r="M67" s="17">
@@ -4482,7 +4520,7 @@
         <v>208</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="L68" s="5"/>
       <c r="M68" s="5">
@@ -4511,7 +4549,7 @@
       <c r="I69" s="18"/>
       <c r="J69" s="18"/>
       <c r="K69" s="18" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="L69" s="18"/>
       <c r="M69" s="17">
@@ -4546,7 +4584,7 @@
         <v>208</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="L70" s="5"/>
       <c r="M70" s="5">
@@ -4575,7 +4613,7 @@
       <c r="I71" s="18"/>
       <c r="J71" s="18"/>
       <c r="K71" s="18" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="L71" s="18"/>
       <c r="M71" s="17">
@@ -4610,7 +4648,7 @@
         <v>208</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="L72" s="5"/>
       <c r="M72" s="5">
@@ -4639,7 +4677,7 @@
       <c r="I73" s="18"/>
       <c r="J73" s="18"/>
       <c r="K73" s="18" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="L73" s="18"/>
       <c r="M73" s="17">
@@ -4674,7 +4712,7 @@
         <v>208</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="L74" s="5"/>
       <c r="M74" s="5">
@@ -4705,7 +4743,7 @@
       <c r="I75" s="18"/>
       <c r="J75" s="18"/>
       <c r="K75" s="18" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="L75" s="18"/>
       <c r="M75" s="17">
@@ -4740,7 +4778,7 @@
         <v>212</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="L76" s="5"/>
       <c r="M76" s="5">
@@ -4771,7 +4809,7 @@
       <c r="I77" s="18"/>
       <c r="J77" s="18"/>
       <c r="K77" s="18" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="L77" s="18"/>
       <c r="M77" s="17">
@@ -4806,7 +4844,7 @@
         <v>212</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="L78" s="5"/>
       <c r="M78" s="5">
@@ -4821,10 +4859,10 @@
         <v>230</v>
       </c>
       <c r="C79" s="18" t="s">
-        <v>297</v>
+        <v>553</v>
       </c>
       <c r="D79" s="18" t="s">
-        <v>298</v>
+        <v>554</v>
       </c>
       <c r="E79" s="21"/>
       <c r="F79" s="17" t="s">
@@ -4834,9 +4872,7 @@
       <c r="H79" s="18"/>
       <c r="I79" s="18"/>
       <c r="J79" s="18"/>
-      <c r="K79" s="18" t="s">
-        <v>441</v>
-      </c>
+      <c r="K79" s="18"/>
       <c r="L79" s="18"/>
       <c r="M79" s="17">
         <v>9</v>
@@ -4870,7 +4906,7 @@
         <v>213</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="L80" s="5"/>
       <c r="M80" s="5">
@@ -4899,7 +4935,7 @@
       <c r="I81" s="18"/>
       <c r="J81" s="18"/>
       <c r="K81" s="18" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="L81" s="18"/>
       <c r="M81" s="17">
@@ -4934,7 +4970,7 @@
         <v>213</v>
       </c>
       <c r="K82" s="22" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="L82" s="22"/>
       <c r="M82" s="22">
@@ -4963,7 +4999,7 @@
       <c r="I83" s="10"/>
       <c r="J83" s="10"/>
       <c r="K83" s="10" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="L83" s="10"/>
       <c r="M83" s="9">
@@ -4998,7 +5034,7 @@
         <v>213</v>
       </c>
       <c r="K84" s="8" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="L84" s="8"/>
       <c r="M84" s="8">
@@ -5027,7 +5063,7 @@
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
       <c r="K85" s="10" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="L85" s="10"/>
       <c r="M85" s="9">
@@ -5059,9 +5095,7 @@
       <c r="J86" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="K86" s="8" t="s">
-        <v>448</v>
-      </c>
+      <c r="K86" s="8"/>
       <c r="L86" s="8" t="s">
         <v>306</v>
       </c>
@@ -5097,7 +5131,7 @@
         <v>217</v>
       </c>
       <c r="K87" s="6" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="L87" s="6"/>
       <c r="M87" s="6">
@@ -5128,7 +5162,7 @@
       <c r="I88" s="10"/>
       <c r="J88" s="10"/>
       <c r="K88" s="10" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="L88" s="10"/>
       <c r="M88" s="9">
@@ -5163,7 +5197,7 @@
         <v>217</v>
       </c>
       <c r="K89" s="6" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="L89" s="6"/>
       <c r="M89" s="6">
@@ -5194,7 +5228,7 @@
       <c r="I90" s="10"/>
       <c r="J90" s="10"/>
       <c r="K90" s="10" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="L90" s="10"/>
       <c r="M90" s="9">
@@ -5224,9 +5258,7 @@
       <c r="H91" s="10"/>
       <c r="I91" s="10"/>
       <c r="J91" s="10"/>
-      <c r="K91" s="10" t="s">
-        <v>453</v>
-      </c>
+      <c r="K91" s="10"/>
       <c r="L91" s="10" t="s">
         <v>301</v>
       </c>
@@ -5262,7 +5294,7 @@
         <v>217</v>
       </c>
       <c r="K92" s="6" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="L92" s="6"/>
       <c r="M92" s="6">
@@ -5293,7 +5325,7 @@
       <c r="I93" s="10"/>
       <c r="J93" s="10"/>
       <c r="K93" s="10" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="L93" s="10"/>
       <c r="M93" s="9">
@@ -5328,7 +5360,7 @@
         <v>218</v>
       </c>
       <c r="K94" s="6" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="L94" s="6"/>
       <c r="M94" s="6">
@@ -5359,7 +5391,7 @@
       <c r="I95" s="10"/>
       <c r="J95" s="10"/>
       <c r="K95" s="10" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="L95" s="10"/>
       <c r="M95" s="9">
@@ -5394,7 +5426,7 @@
         <v>218</v>
       </c>
       <c r="K96" s="6" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="L96" s="6"/>
       <c r="M96" s="6">
@@ -5425,7 +5457,7 @@
       <c r="I97" s="10"/>
       <c r="J97" s="10"/>
       <c r="K97" s="10" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="L97" s="10"/>
       <c r="M97" s="9">
@@ -5460,7 +5492,7 @@
         <v>221</v>
       </c>
       <c r="K98" s="6" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="L98" s="6"/>
       <c r="M98" s="6">
@@ -5491,7 +5523,7 @@
       <c r="I99" s="10"/>
       <c r="J99" s="10"/>
       <c r="K99" s="10" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="L99" s="10"/>
       <c r="M99" s="9">
@@ -5526,7 +5558,7 @@
         <v>221</v>
       </c>
       <c r="K100" s="6" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="L100" s="6"/>
       <c r="M100" s="6">
@@ -5561,7 +5593,7 @@
         <v>223</v>
       </c>
       <c r="K101" s="6" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="L101" s="6"/>
       <c r="M101" s="6">
@@ -5592,7 +5624,7 @@
       <c r="I102" s="10"/>
       <c r="J102" s="10"/>
       <c r="K102" s="10" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="L102" s="10"/>
       <c r="M102" s="9">
@@ -5627,7 +5659,7 @@
         <v>223</v>
       </c>
       <c r="K103" s="6" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="L103" s="6"/>
       <c r="M103" s="6">
@@ -5642,23 +5674,23 @@
         <v>242</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>186</v>
+        <v>293</v>
       </c>
       <c r="D104" s="10" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E104" s="9"/>
       <c r="F104" s="9" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G104" s="9">
-        <v>1983</v>
+        <v>1972</v>
       </c>
       <c r="H104" s="10"/>
       <c r="I104" s="10"/>
       <c r="J104" s="10"/>
       <c r="K104" s="10" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="L104" s="10"/>
       <c r="M104" s="9">
@@ -5693,7 +5725,7 @@
         <v>223</v>
       </c>
       <c r="K105" s="6" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="L105" s="6"/>
       <c r="M105" s="6">
@@ -5708,23 +5740,23 @@
         <v>241</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>293</v>
+        <v>186</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E106" s="9"/>
       <c r="F106" s="9" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G106" s="9">
-        <v>1972</v>
+        <v>1983</v>
       </c>
       <c r="H106" s="10"/>
       <c r="I106" s="10"/>
       <c r="J106" s="10"/>
       <c r="K106" s="10" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="L106" s="10"/>
       <c r="M106" s="9">
@@ -5759,7 +5791,7 @@
         <v>224</v>
       </c>
       <c r="K107" s="6" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="L107" s="6"/>
       <c r="M107" s="6">
@@ -5790,7 +5822,7 @@
       <c r="I108" s="10"/>
       <c r="J108" s="10"/>
       <c r="K108" s="10" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
       <c r="L108" s="10"/>
       <c r="M108" s="9">
@@ -5825,7 +5857,7 @@
         <v>224</v>
       </c>
       <c r="K109" s="6" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="L109" s="6"/>
       <c r="M109" s="6">
@@ -5860,7 +5892,7 @@
         <v>228</v>
       </c>
       <c r="K110" s="6" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="L110" s="6"/>
       <c r="M110" s="6">
@@ -5895,7 +5927,7 @@
         <v>228</v>
       </c>
       <c r="K111" s="6" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="L111" s="6"/>
       <c r="M111" s="6">
@@ -5930,7 +5962,7 @@
         <v>229</v>
       </c>
       <c r="K112" s="6" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="L112" s="6"/>
       <c r="M112" s="6">
@@ -5965,7 +5997,7 @@
         <v>229</v>
       </c>
       <c r="K113" s="6" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="L113" s="6"/>
       <c r="M113" s="6">
@@ -5998,7 +6030,7 @@
         <v>231</v>
       </c>
       <c r="K114" s="6" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="L114" s="6"/>
       <c r="M114" s="6">
@@ -6031,7 +6063,7 @@
         <v>231</v>
       </c>
       <c r="K115" s="6" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="L115" s="6"/>
       <c r="M115" s="6">
@@ -6066,7 +6098,7 @@
         <v>232</v>
       </c>
       <c r="K116" s="6" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="L116" s="6"/>
       <c r="M116" s="6">
@@ -6099,7 +6131,7 @@
         <v>232</v>
       </c>
       <c r="K117" s="6" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="L117" s="6"/>
       <c r="M117" s="6">
@@ -6132,7 +6164,7 @@
         <v>232</v>
       </c>
       <c r="K118" s="6" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
       <c r="L118" s="6"/>
       <c r="M118" s="6">
@@ -6167,7 +6199,7 @@
         <v>234</v>
       </c>
       <c r="K119" s="6" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="L119" s="6"/>
       <c r="M119" s="6">
@@ -6202,7 +6234,7 @@
         <v>234</v>
       </c>
       <c r="K120" s="6" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="L120" s="6"/>
       <c r="M120" s="6">
@@ -6237,7 +6269,7 @@
         <v>299</v>
       </c>
       <c r="K121" s="6" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="L121" s="6"/>
       <c r="M121" s="6">
@@ -6272,7 +6304,7 @@
         <v>235</v>
       </c>
       <c r="K122" s="6" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
       <c r="L122" s="6"/>
       <c r="M122" s="6">
@@ -6307,7 +6339,7 @@
         <v>237</v>
       </c>
       <c r="K123" s="6" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="L123" s="6"/>
       <c r="M123" s="6">
@@ -6342,7 +6374,7 @@
         <v>237</v>
       </c>
       <c r="K124" s="6" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="L124" s="6"/>
       <c r="M124" s="6">
@@ -6377,7 +6409,7 @@
         <v>240</v>
       </c>
       <c r="K125" s="6" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="L125" s="6"/>
       <c r="M125" s="6">
@@ -6412,7 +6444,7 @@
         <v>240</v>
       </c>
       <c r="K126" s="6" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="L126" s="6"/>
       <c r="M126" s="6">
@@ -6443,7 +6475,7 @@
       <c r="I127" s="10"/>
       <c r="J127" s="10"/>
       <c r="K127" s="13" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="L127" s="10"/>
       <c r="M127" s="9">
@@ -6478,7 +6510,7 @@
         <v>242</v>
       </c>
       <c r="K128" s="6" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="L128" s="6"/>
       <c r="M128" s="6">
@@ -6513,7 +6545,7 @@
         <v>242</v>
       </c>
       <c r="K129" s="6" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="L129" s="6"/>
       <c r="M129" s="6">
@@ -6548,7 +6580,7 @@
         <v>243</v>
       </c>
       <c r="K130" s="6" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="L130" s="6"/>
       <c r="M130" s="6">
@@ -6583,7 +6615,7 @@
         <v>243</v>
       </c>
       <c r="K131" s="6" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="L131" s="6"/>
       <c r="M131" s="6">
@@ -7104,27 +7136,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>323</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="30" t="s">
         <v>324</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>382</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>325</v>
       </c>
       <c r="E1" s="25" t="s">
         <v>380</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>536</v>
+        <v>530</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="7" t="s">
@@ -7134,7 +7166,7 @@
         <v>379</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>381</v>
@@ -7144,17 +7176,17 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="7" t="s">
         <v>326</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>498</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>499</v>
+        <v>492</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>493</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>381</v>
@@ -7164,17 +7196,17 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="7" t="s">
         <v>326</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>540</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>541</v>
+        <v>534</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>535</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>381</v>
@@ -7184,17 +7216,17 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>534</v>
-      </c>
-      <c r="D5" s="29" t="s">
-        <v>535</v>
+      <c r="C5" s="7" t="s">
+        <v>528</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>529</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>381</v>
@@ -7204,17 +7236,17 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C6" s="29" t="s">
-        <v>509</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>510</v>
+      <c r="C6" s="7" t="s">
+        <v>503</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>504</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>381</v>
@@ -7224,17 +7256,17 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>528</v>
-      </c>
-      <c r="C7" s="29" t="s">
-        <v>529</v>
-      </c>
-      <c r="D7" s="29" t="s">
-        <v>530</v>
+      <c r="B7" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>523</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>524</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>381</v>
@@ -7244,7 +7276,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -7254,7 +7286,7 @@
         <v>384</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>517</v>
+        <v>511</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>381</v>
@@ -7264,7 +7296,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="7" t="s">
         <v>207</v>
       </c>
       <c r="B9" s="7" t="s">
@@ -7274,7 +7306,7 @@
         <v>383</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>381</v>
@@ -7284,8 +7316,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="29" t="s">
-        <v>47</v>
+      <c r="A10" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>326</v>
@@ -7294,7 +7326,7 @@
         <v>385</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>512</v>
+        <v>506</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>381</v>
@@ -7304,7 +7336,7 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B11" s="7" t="s">
@@ -7314,7 +7346,7 @@
         <v>386</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>381</v>
@@ -7324,7 +7356,7 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="7" t="s">
         <v>65</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -7334,7 +7366,7 @@
         <v>327</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>511</v>
+        <v>505</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>381</v>
@@ -7344,17 +7376,17 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="7" t="s">
         <v>42</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>326</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>514</v>
+        <v>508</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>381</v>
@@ -7364,17 +7396,17 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="29" t="s">
-        <v>501</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>502</v>
+      <c r="C14" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>496</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>381</v>
@@ -7384,17 +7416,17 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>513</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>524</v>
+      <c r="C15" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>518</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>381</v>
@@ -7404,17 +7436,17 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="7" t="s">
         <v>310</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>326</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>538</v>
+        <v>532</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>381</v>
@@ -7424,17 +7456,17 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="7" t="s">
         <v>326</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>515</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>516</v>
+        <v>509</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>510</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>381</v>
@@ -7444,17 +7476,17 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C18" s="29" t="s">
-        <v>518</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>519</v>
+      <c r="C18" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>513</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>381</v>
@@ -7464,17 +7496,17 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="32" t="s">
+      <c r="A19" s="24" t="s">
         <v>208</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C19" s="29" t="s">
-        <v>520</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>523</v>
+      <c r="C19" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>517</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>381</v>
@@ -7484,17 +7516,17 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="32" t="s">
+      <c r="A20" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="C20" s="29" t="s">
-        <v>521</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>522</v>
+      <c r="C20" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>516</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>381</v>
@@ -7511,10 +7543,10 @@
         <v>326</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>546</v>
+        <v>540</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>381</v>
@@ -7586,7 +7618,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2870D094-0F04-43A9-85F0-3281621B51DF}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -7621,10 +7653,10 @@
         <v>389</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="D2" t="s">
-        <v>553</v>
+        <v>547</v>
       </c>
       <c r="E2" t="s">
         <v>347</v>
@@ -7638,7 +7670,7 @@
         <v>389</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="D3" t="s">
         <v>390</v>
@@ -7655,10 +7687,10 @@
         <v>389</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="D4" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="E4" t="s">
         <v>347</v>
@@ -7672,7 +7704,7 @@
         <v>389</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="D5" t="s">
         <v>390</v>
@@ -7689,10 +7721,10 @@
         <v>389</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="D6" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="E6" t="s">
         <v>347</v>
@@ -7706,10 +7738,10 @@
         <v>389</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="D7" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="E7" t="s">
         <v>347</v>
@@ -7723,10 +7755,10 @@
         <v>389</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="D8" t="s">
-        <v>552</v>
+        <v>546</v>
       </c>
       <c r="E8" t="s">
         <v>347</v>
@@ -7740,10 +7772,10 @@
         <v>389</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>557</v>
+        <v>551</v>
       </c>
       <c r="D9" t="s">
-        <v>558</v>
+        <v>552</v>
       </c>
       <c r="E9" t="s">
         <v>347</v>
@@ -7757,12 +7789,46 @@
         <v>389</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="D10" t="s">
+        <v>550</v>
+      </c>
+      <c r="E10" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>389</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>555</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
+        <v>558</v>
+      </c>
+      <c r="E11" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>389</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="E10" t="s">
+      <c r="D12" t="s">
+        <v>557</v>
+      </c>
+      <c r="E12" t="s">
         <v>347</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update about theo .md
</commit_message>
<xml_diff>
--- a/data/DATA_GIAPHA.xlsx
+++ b/data/DATA_GIAPHA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\giapha\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2FA415-BBA5-4729-9005-DBC981CC408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31819BCC-73DF-44EC-A6C8-0EFAC02B7A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{82229A43-EBB1-44A5-B6DE-F008EE3D4237}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82229A43-EBB1-44A5-B6DE-F008EE3D4237}"/>
   </bookViews>
   <sheets>
     <sheet name="PERSONS" sheetId="1" r:id="rId1"/>
@@ -6504,10 +6504,10 @@
       </c>
       <c r="H128" s="6"/>
       <c r="I128" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J128" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K128" s="6" t="s">
         <v>484</v>
@@ -6539,10 +6539,10 @@
       </c>
       <c r="H129" s="6"/>
       <c r="I129" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J129" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K129" s="6" t="s">
         <v>485</v>

</xml_diff>